<commit_message>
Update MigratedStores tracking sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/MigratedStores.xlsx
+++ b/Docs/MigratedStores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ProjectsGIT\PawnProFB\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23A200F7-BB64-4135-822E-A6CEC37139AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF64118-878C-48BA-9546-56AAA12B2BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C89F38F1-ECC2-4536-B6D8-36FB7ABEFE69}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Perez Cash II</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t>When</t>
+  </si>
+  <si>
+    <t>11048 W. Flagler St</t>
+  </si>
+  <si>
+    <t>Ricardo Joyeria</t>
   </si>
 </sst>
 </file>
@@ -142,10 +148,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,12 +487,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{237F7F61-BA31-4C5A-9228-BDF65D551602}">
-  <dimension ref="B1:H10"/>
+  <dimension ref="B1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="16.7109375" customWidth="1"/>
     <col min="5" max="5" width="32.85546875" customWidth="1"/>
     <col min="6" max="6" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -535,44 +543,64 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" s="3">
+        <v>46223</v>
+      </c>
+    </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H6" s="2">
-        <v>46249</v>
-      </c>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="2">
+        <v>46249</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
         <v>16</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F8" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
         <v>12</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E11" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>